<commit_message>
feat: update version to 1.3.4 and improve price calculations in emissions.py
</commit_message>
<xml_diff>
--- a/botCTE/botCTE/Alíquota.xlsx
+++ b/botCTE/botCTE/Alíquota.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29930"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brian Marques\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{078037D6-CD6C-4CFD-9F08-81BA3DBE324A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8DE63B0-4877-4DAD-B73D-945B72E26681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AA807991-941E-477F-BBBF-867C6D8017B1}"/>
   </bookViews>
@@ -129,7 +129,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -397,9 +397,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -437,7 +437,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -543,7 +543,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -685,7 +685,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -694,14 +694,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6596CEC0-C1AD-42F0-9A7D-CB3E5481D5E4}">
   <dimension ref="A1:AC28"/>
-  <sheetFormatPr defaultColWidth="4.140625" defaultRowHeight="17.25" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="4.140625" defaultRowHeight="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" style="17"/>
     <col min="2" max="28" width="5.5703125" style="18" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="4.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="1" customFormat="1" ht="17.25" customHeight="1" thickBot="1">
+    <row r="1" spans="1:29" s="1" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -788,7 +788,7 @@
       </c>
       <c r="AC1" s="2"/>
     </row>
-    <row r="2" spans="1:29" ht="17.25" customHeight="1">
+    <row r="2" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
@@ -874,7 +874,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:29" ht="17.25" customHeight="1">
+    <row r="3" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
@@ -882,7 +882,7 @@
         <v>12</v>
       </c>
       <c r="C3" s="5">
-        <v>20</v>
+        <v>20.5</v>
       </c>
       <c r="D3" s="12">
         <v>12</v>
@@ -960,7 +960,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:29" ht="17.25" customHeight="1">
+    <row r="4" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
@@ -1046,7 +1046,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:29" ht="17.25" customHeight="1">
+    <row r="5" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
@@ -1132,7 +1132,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:29" ht="17.25" customHeight="1">
+    <row r="6" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>5</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:29" ht="17.25" customHeight="1">
+    <row r="7" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
@@ -1304,7 +1304,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:29" ht="17.25" customHeight="1">
+    <row r="8" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>7</v>
       </c>
@@ -1390,7 +1390,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:29" ht="17.25" customHeight="1">
+    <row r="9" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>8</v>
       </c>
@@ -1476,7 +1476,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:29" ht="17.25" customHeight="1">
+    <row r="10" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>9</v>
       </c>
@@ -1562,7 +1562,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:29" ht="17.25" customHeight="1">
+    <row r="11" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>10</v>
       </c>
@@ -1648,7 +1648,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:29" ht="17.25" customHeight="1">
+    <row r="12" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>11</v>
       </c>
@@ -1734,7 +1734,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:29" ht="17.25" customHeight="1">
+    <row r="13" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>12</v>
       </c>
@@ -1820,7 +1820,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:29" ht="17.25" customHeight="1">
+    <row r="14" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>13</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:29" ht="17.25" customHeight="1">
+    <row r="15" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>14</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:29" ht="17.25" customHeight="1">
+    <row r="16" spans="1:29" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>15</v>
       </c>
@@ -2078,7 +2078,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="17.25" customHeight="1">
+    <row r="17" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>16</v>
       </c>
@@ -2164,7 +2164,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="17.25" customHeight="1">
+    <row r="18" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>17</v>
       </c>
@@ -2250,7 +2250,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="17.25" customHeight="1">
+    <row r="19" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>18</v>
       </c>
@@ -2336,7 +2336,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="17.25" customHeight="1">
+    <row r="20" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>19</v>
       </c>
@@ -2422,7 +2422,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="17.25" customHeight="1">
+    <row r="21" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>20</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="17.25" customHeight="1">
+    <row r="22" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>21</v>
       </c>
@@ -2594,7 +2594,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="17.25" customHeight="1">
+    <row r="23" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>22</v>
       </c>
@@ -2680,7 +2680,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="17.25" customHeight="1">
+    <row r="24" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>23</v>
       </c>
@@ -2766,7 +2766,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="17.25" customHeight="1">
+    <row r="25" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>24</v>
       </c>
@@ -2852,7 +2852,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="17.25" customHeight="1">
+    <row r="26" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>25</v>
       </c>
@@ -2938,7 +2938,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:28" ht="17.25" customHeight="1">
+    <row r="27" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>26</v>
       </c>
@@ -3024,7 +3024,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="17.25" customHeight="1" thickBot="1">
+    <row r="28" spans="1:28" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
         <v>27</v>
       </c>

</xml_diff>